<commit_message>
docs: 精度验收标准.xlsx 移除 minimax-m3 列
</commit_message>
<xml_diff>
--- a/精度验收标准.xlsx
+++ b/精度验收标准.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -482,8 +482,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -521,15 +520,10 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>minimax-m3</t>
+          <t>hy4-preview</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>hy4-preview</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>浮动范围</t>
         </is>
@@ -556,12 +550,9 @@
         <v>95.67</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>95.67</v>
-      </c>
-      <c r="G3" s="4" t="n">
         <v>96</v>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -588,12 +579,9 @@
         <v>32.35</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>32.35</v>
-      </c>
-      <c r="G4" s="4" t="n">
         <v>34.33</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -620,12 +608,9 @@
         <v>87.25</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="G5" s="4" t="n">
         <v>85.95999999999999</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -652,12 +637,9 @@
         <v>37.56</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>37.56</v>
-      </c>
-      <c r="G6" s="4" t="n">
         <v>33.7</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -684,12 +666,9 @@
         <v>89.73</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>89.73</v>
-      </c>
-      <c r="G7" s="4" t="n">
         <v>94.44</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -716,12 +695,9 @@
         <v>68.89</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>68.89</v>
-      </c>
-      <c r="G8" s="4" t="n">
         <v>67.56</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -748,12 +724,9 @@
         <v>87.7</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>87.7</v>
-      </c>
-      <c r="G9" s="4" t="n">
         <v>82.22</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -780,12 +753,9 @@
         <v>98.42</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>98.42</v>
-      </c>
-      <c r="G10" s="4" t="n">
         <v>77.14</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -812,12 +782,9 @@
         <v>68.05</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>68.05</v>
-      </c>
-      <c r="G11" s="4" t="n">
         <v>74.7</v>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -844,12 +811,9 @@
         <v>88.7</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="G12" s="4" t="n">
         <v>77.27</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -879,15 +843,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>86.92</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -919,15 +878,10 @@
           <t>-</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>85.42</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>±2-4%</t>
         </is>
@@ -942,8 +896,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>